<commit_message>
Regenerar datos con fix de moneda nativa; alias derivados del ETL (plan/canal/cliente); base SQLite poblada
</commit_message>
<xml_diff>
--- a/data/raw/contratos/contratos.xlsx
+++ b/data/raw/contratos/contratos.xlsx
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>906430</v>
+        <v>230</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>915170</v>
+        <v>230</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>905050</v>
+        <v>230</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>917240</v>
+        <v>230</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>919080</v>
+        <v>230</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>930120</v>
+        <v>230</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1411,7 +1411,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>917240</v>
+        <v>230</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1640,7 +1640,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>915170</v>
+        <v>230</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>929430</v>
+        <v>230</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1929,7 +1929,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>901830</v>
+        <v>230</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>930120</v>
+        <v>230</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>

</xml_diff>